<commit_message>
full height data from 3/23/26
</commit_message>
<xml_diff>
--- a/height_data.xlsx
+++ b/height_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jacksonstrand/Documents/GitHub/Linaria_specProj/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{806A1CD9-7B11-6D48-BF1D-30CCBACAC980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{578A45BC-1BD2-AA4D-865C-783A34B81A5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="5" xr2:uid="{8DE00727-C8D7-6A48-9276-98A4664605B4}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="92">
   <si>
     <t>lc1</t>
   </si>
@@ -5454,7 +5454,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35664989-61A4-F94C-A05A-9E3D17A531B3}">
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="10.1640625" bestFit="1" customWidth="1"/>
@@ -6226,6 +6226,292 @@
       <c r="C32">
         <v>0</v>
       </c>
+      <c r="D32">
+        <v>62.8</v>
+      </c>
+      <c r="E32" s="2">
+        <v>45.1</v>
+      </c>
+      <c r="F32" s="2">
+        <v>45.7</v>
+      </c>
+      <c r="G32" s="2">
+        <v>54.4</v>
+      </c>
+      <c r="H32" s="2">
+        <v>54.2</v>
+      </c>
+      <c r="I32" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="J32" s="2">
+        <v>48.6</v>
+      </c>
+    </row>
+    <row r="33" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B33" t="s">
+        <v>15</v>
+      </c>
+      <c r="C33">
+        <v>0</v>
+      </c>
+      <c r="D33">
+        <v>8</v>
+      </c>
+      <c r="E33" s="2">
+        <v>23.9</v>
+      </c>
+      <c r="F33" s="2">
+        <v>17.100000000000001</v>
+      </c>
+      <c r="G33" s="2">
+        <v>40.799999999999997</v>
+      </c>
+      <c r="H33" s="2">
+        <v>4.2</v>
+      </c>
+      <c r="I33" s="2">
+        <v>5.5</v>
+      </c>
+      <c r="J33" s="2">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="K33" s="2">
+        <v>25.6</v>
+      </c>
+      <c r="L33" s="2">
+        <v>1.7</v>
+      </c>
+      <c r="O33" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="34" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B34" t="s">
+        <v>13</v>
+      </c>
+      <c r="C34">
+        <v>1</v>
+      </c>
+      <c r="D34">
+        <v>66</v>
+      </c>
+      <c r="E34" s="2">
+        <v>26.2</v>
+      </c>
+      <c r="F34" s="2">
+        <v>31.6</v>
+      </c>
+      <c r="G34" s="2">
+        <v>48.6</v>
+      </c>
+      <c r="H34" s="2">
+        <v>62.4</v>
+      </c>
+      <c r="I34" s="2">
+        <v>68.400000000000006</v>
+      </c>
+      <c r="J34" s="2">
+        <v>31.1</v>
+      </c>
+      <c r="K34" s="2">
+        <v>44.4</v>
+      </c>
+      <c r="L34" s="2">
+        <v>31.9</v>
+      </c>
+      <c r="M34" s="2">
+        <v>43.6</v>
+      </c>
+      <c r="N34" s="2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="35" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B35" t="s">
+        <v>10</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
+      </c>
+      <c r="D35">
+        <v>58.5</v>
+      </c>
+      <c r="E35" s="2">
+        <v>48.5</v>
+      </c>
+      <c r="F35" s="2">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="G35" s="2">
+        <v>8</v>
+      </c>
+      <c r="H35" s="2">
+        <v>11.6</v>
+      </c>
+      <c r="I35" s="2">
+        <v>65</v>
+      </c>
+      <c r="J35" s="2">
+        <v>2.5</v>
+      </c>
+      <c r="K35" s="2">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="36" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B36" t="s">
+        <v>12</v>
+      </c>
+      <c r="C36">
+        <v>0</v>
+      </c>
+      <c r="D36">
+        <v>60.2</v>
+      </c>
+      <c r="E36" s="2">
+        <v>58.5</v>
+      </c>
+      <c r="F36" s="2">
+        <v>33.6</v>
+      </c>
+      <c r="G36" s="2">
+        <v>52.2</v>
+      </c>
+      <c r="H36" s="2">
+        <v>39.4</v>
+      </c>
+      <c r="I36" s="2">
+        <v>38.700000000000003</v>
+      </c>
+      <c r="J36" s="2">
+        <v>46.7</v>
+      </c>
+      <c r="K36" s="2">
+        <v>66</v>
+      </c>
+      <c r="L36" s="2">
+        <v>26.3</v>
+      </c>
+      <c r="M36" s="2">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="37" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B37" t="s">
+        <v>6</v>
+      </c>
+      <c r="C37">
+        <v>1</v>
+      </c>
+      <c r="D37">
+        <v>10.199999999999999</v>
+      </c>
+      <c r="E37" s="2">
+        <v>31.1</v>
+      </c>
+      <c r="F37" s="2">
+        <v>14</v>
+      </c>
+      <c r="G37" s="2">
+        <v>50.8</v>
+      </c>
+      <c r="H37" s="2">
+        <v>32.799999999999997</v>
+      </c>
+      <c r="I37" s="2">
+        <v>2.4</v>
+      </c>
+      <c r="J37" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="K37" s="2">
+        <v>7.7</v>
+      </c>
+      <c r="O37" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="38" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B38" t="s">
+        <v>36</v>
+      </c>
+      <c r="C38">
+        <v>1</v>
+      </c>
+      <c r="D38">
+        <v>59</v>
+      </c>
+      <c r="E38" s="2">
+        <v>30.4</v>
+      </c>
+      <c r="F38" s="2">
+        <v>50.1</v>
+      </c>
+      <c r="G38" s="2">
+        <v>48.8</v>
+      </c>
+      <c r="H38" s="2">
+        <v>37.6</v>
+      </c>
+      <c r="I38" s="2">
+        <v>58.1</v>
+      </c>
+      <c r="J38" s="2">
+        <v>42.2</v>
+      </c>
+      <c r="K38" s="2">
+        <v>12.9</v>
+      </c>
+    </row>
+    <row r="39" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B39" t="s">
+        <v>0</v>
+      </c>
+      <c r="C39">
+        <v>0</v>
+      </c>
+      <c r="D39">
+        <v>52.4</v>
+      </c>
+      <c r="E39" s="2">
+        <v>51.6</v>
+      </c>
+      <c r="F39" s="2">
+        <v>47.4</v>
+      </c>
+      <c r="G39" s="2">
+        <v>46.1</v>
+      </c>
+      <c r="H39" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="I39" s="2">
+        <v>7.6</v>
+      </c>
+      <c r="J39" s="2">
+        <v>13.5</v>
+      </c>
+      <c r="K39" s="2">
+        <v>4.5</v>
+      </c>
+      <c r="L39" s="2">
+        <v>10.6</v>
+      </c>
+    </row>
+    <row r="40" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B40" t="s">
+        <v>3</v>
+      </c>
+      <c r="C40">
+        <v>0</v>
+      </c>
+      <c r="D40">
+        <v>79.099999999999994</v>
+      </c>
+      <c r="E40" s="2">
+        <v>26.8</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>